<commit_message>
survey completed harassment branch version
</commit_message>
<xml_diff>
--- a/questionnaire/survey_results.xlsx
+++ b/questionnaire/survey_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R4"/>
+  <dimension ref="A1:R7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -658,9 +658,6 @@
           <t>2026-03-05 06:52:16</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>週2休</t>
@@ -722,6 +719,160 @@
         </is>
       </c>
       <c r="R4" t="inlineStr">
+        <is>
+          <t>テスト</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-03-05 15:22:51</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>on</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>on</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>on</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>on</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-03-06 00:25:02</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>on</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>on</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>on</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-03-06 00:42:37</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>on</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>on</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>on</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>テスト</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
         <is>
           <t>テスト</t>
         </is>

</xml_diff>

<commit_message>
fix numeric survey values
</commit_message>
<xml_diff>
--- a/questionnaire/survey_results.xlsx
+++ b/questionnaire/survey_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:R10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -824,9 +824,6 @@
           <t>2026-03-06 00:42:37</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>on</t>
@@ -873,6 +870,170 @@
         </is>
       </c>
       <c r="R7" t="inlineStr">
+        <is>
+          <t>テスト</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-03-06 06:06:35</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>テスト</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>テスト</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-03-06 06:11:21</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>テスト</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>テスト</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-03-06 07:00:53</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>テスト</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
         <is>
           <t>テスト</t>
         </is>

</xml_diff>